<commit_message>
organized workflow into phases
</commit_message>
<xml_diff>
--- a/data/nh_to_cluster.xlsx
+++ b/data/nh_to_cluster.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/renudinesh/Final-Project/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1814F314-BA56-AF4A-8465-94664CDE1533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B285ECA0-DD4F-E44E-A401-238F3CFC9BB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="167">
   <si>
-    <t>AREA_NAME</t>
+    <t>Neighbourhood</t>
   </si>
   <si>
     <t>ClusterName</t>
@@ -514,32 +514,26 @@
     <t>North York</t>
   </si>
   <si>
-    <t>Black Creek/Humber Summit &amp; York Weston Pelham</t>
-  </si>
-  <si>
     <t>Downtown East &amp; Downtown West</t>
   </si>
   <si>
     <t>North Etobicoke &amp; South Etobicoke</t>
+  </si>
+  <si>
+    <t>Black Creek/ Humber Summit &amp; York Weston Pelham</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -558,7 +552,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -566,31 +560,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -900,7 +876,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
@@ -925,7 +901,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -1029,7 +1005,7 @@
         <v>17</v>
       </c>
       <c r="B17" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -1077,7 +1053,7 @@
         <v>23</v>
       </c>
       <c r="B23" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
@@ -1109,7 +1085,7 @@
         <v>27</v>
       </c>
       <c r="B27" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
@@ -1181,7 +1157,7 @@
         <v>36</v>
       </c>
       <c r="B36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
@@ -1197,7 +1173,7 @@
         <v>38</v>
       </c>
       <c r="B38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
@@ -1205,7 +1181,7 @@
         <v>39</v>
       </c>
       <c r="B39" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
@@ -1253,7 +1229,7 @@
         <v>45</v>
       </c>
       <c r="B45" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
@@ -1269,7 +1245,7 @@
         <v>47</v>
       </c>
       <c r="B47" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
@@ -1277,7 +1253,7 @@
         <v>48</v>
       </c>
       <c r="B48" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -1285,7 +1261,7 @@
         <v>49</v>
       </c>
       <c r="B49" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
@@ -1325,7 +1301,7 @@
         <v>54</v>
       </c>
       <c r="B54" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
@@ -1365,7 +1341,7 @@
         <v>59</v>
       </c>
       <c r="B59" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
@@ -1413,7 +1389,7 @@
         <v>65</v>
       </c>
       <c r="B65" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
@@ -1429,7 +1405,7 @@
         <v>67</v>
       </c>
       <c r="B67" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
@@ -1437,7 +1413,7 @@
         <v>68</v>
       </c>
       <c r="B68" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
@@ -1461,7 +1437,7 @@
         <v>71</v>
       </c>
       <c r="B71" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
@@ -1501,7 +1477,7 @@
         <v>76</v>
       </c>
       <c r="B76" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
@@ -1509,7 +1485,7 @@
         <v>77</v>
       </c>
       <c r="B77" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
@@ -1517,7 +1493,7 @@
         <v>78</v>
       </c>
       <c r="B78" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
@@ -1573,7 +1549,7 @@
         <v>85</v>
       </c>
       <c r="B85" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
@@ -1581,7 +1557,7 @@
         <v>86</v>
       </c>
       <c r="B86" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
@@ -1613,7 +1589,7 @@
         <v>90</v>
       </c>
       <c r="B90" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
@@ -1629,7 +1605,7 @@
         <v>92</v>
       </c>
       <c r="B92" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
@@ -1653,7 +1629,7 @@
         <v>95</v>
       </c>
       <c r="B95" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
@@ -1685,7 +1661,7 @@
         <v>99</v>
       </c>
       <c r="B99" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
@@ -1789,7 +1765,7 @@
         <v>112</v>
       </c>
       <c r="B112" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.2">
@@ -1813,7 +1789,7 @@
         <v>115</v>
       </c>
       <c r="B115" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
@@ -1821,7 +1797,7 @@
         <v>116</v>
       </c>
       <c r="B116" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
@@ -1829,7 +1805,7 @@
         <v>117</v>
       </c>
       <c r="B117" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
@@ -1893,7 +1869,7 @@
         <v>125</v>
       </c>
       <c r="B125" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="126" spans="1:2" x14ac:dyDescent="0.2">
@@ -1901,7 +1877,7 @@
         <v>126</v>
       </c>
       <c r="B126" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="127" spans="1:2" x14ac:dyDescent="0.2">
@@ -1909,7 +1885,7 @@
         <v>127</v>
       </c>
       <c r="B127" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="128" spans="1:2" x14ac:dyDescent="0.2">
@@ -1933,7 +1909,7 @@
         <v>130</v>
       </c>
       <c r="B130" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="131" spans="1:2" x14ac:dyDescent="0.2">
@@ -1965,7 +1941,7 @@
         <v>134</v>
       </c>
       <c r="B134" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="135" spans="1:2" x14ac:dyDescent="0.2">
@@ -1981,7 +1957,7 @@
         <v>136</v>
       </c>
       <c r="B136" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="137" spans="1:2" x14ac:dyDescent="0.2">
@@ -1989,7 +1965,7 @@
         <v>137</v>
       </c>
       <c r="B137" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="138" spans="1:2" x14ac:dyDescent="0.2">
@@ -2021,7 +1997,7 @@
         <v>141</v>
       </c>
       <c r="B141" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="142" spans="1:2" x14ac:dyDescent="0.2">
@@ -2029,7 +2005,7 @@
         <v>142</v>
       </c>
       <c r="B142" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="143" spans="1:2" x14ac:dyDescent="0.2">
@@ -2053,7 +2029,7 @@
         <v>145</v>
       </c>
       <c r="B145" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="146" spans="1:2" x14ac:dyDescent="0.2">
@@ -2061,7 +2037,7 @@
         <v>146</v>
       </c>
       <c r="B146" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="147" spans="1:2" x14ac:dyDescent="0.2">
@@ -2085,7 +2061,7 @@
         <v>149</v>
       </c>
       <c r="B149" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="150" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>